<commit_message>
First version html dashboards
</commit_message>
<xml_diff>
--- a/Fichier sivi Stats cce Smart 12 2025.xlsx
+++ b/Fichier sivi Stats cce Smart 12 2025.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rapha\Documents\KPI_Euklead\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rapha\Documents\Smart_Weekly_Helper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D402C2-09D6-438A-BF93-60D2D728EC73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E668456E-9B71-42F5-A607-358170E4A4F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{C3D58F34-A812-5241-9709-533BCCC2C182}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{C3D58F34-A812-5241-9709-533BCCC2C182}"/>
   </bookViews>
   <sheets>
     <sheet name="Base Stats" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4987" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4987" uniqueCount="489">
   <si>
     <t>PORTEFEUILLE 2024</t>
   </si>
@@ -1505,6 +1505,9 @@
   </si>
   <si>
     <t>Analyse Signé</t>
+  </si>
+  <si>
+    <t>Nb de projets correspondant à des catégories Smart+</t>
   </si>
 </sst>
 </file>
@@ -1853,6 +1856,9 @@
     <xf numFmtId="165" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1885,9 +1891,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2224,44 +2227,44 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCCA7716-ECB8-354A-9018-6D10B29DD4DF}">
   <dimension ref="A1:AA408"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="17.3125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.1875" customWidth="1"/>
-    <col min="4" max="4" width="17.1875" customWidth="1"/>
-    <col min="5" max="5" width="28.3125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.6875" customWidth="1"/>
+    <col min="2" max="2" width="17.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.25" customWidth="1"/>
+    <col min="4" max="4" width="17.25" customWidth="1"/>
+    <col min="5" max="5" width="28.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.75" customWidth="1"/>
     <col min="7" max="7" width="8.5" customWidth="1"/>
-    <col min="8" max="8" width="13.3125" customWidth="1"/>
-    <col min="9" max="11" width="14.1875" customWidth="1"/>
-    <col min="12" max="12" width="12.1875" customWidth="1"/>
+    <col min="8" max="8" width="13.375" customWidth="1"/>
+    <col min="9" max="11" width="14.25" customWidth="1"/>
+    <col min="12" max="12" width="12.25" customWidth="1"/>
     <col min="13" max="13" width="17.5" customWidth="1"/>
     <col min="14" max="14" width="23.5" customWidth="1"/>
-    <col min="15" max="15" width="15.8125" customWidth="1"/>
+    <col min="15" max="15" width="15.875" customWidth="1"/>
     <col min="16" max="16" width="9.5" customWidth="1"/>
     <col min="17" max="17" width="17" customWidth="1"/>
-    <col min="18" max="18" width="9.8125" customWidth="1"/>
+    <col min="18" max="18" width="9.875" customWidth="1"/>
     <col min="19" max="19" width="29" customWidth="1"/>
     <col min="22" max="22" width="2" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="2" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.1875" customWidth="1"/>
+    <col min="25" max="25" width="13.25" customWidth="1"/>
     <col min="26" max="26" width="2" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.6875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12.75" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="4.25" bestFit="1" customWidth="1"/>
-    <col min="29" max="32" width="12.3125" bestFit="1" customWidth="1"/>
+    <col min="29" max="32" width="12.375" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="22.625" customWidth="1"/>
     <col min="38" max="38" width="22.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:19" s="2" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:19" s="2" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -2320,7 +2323,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>420</v>
       </c>
@@ -2365,7 +2368,7 @@
       </c>
       <c r="S3" s="6"/>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>406</v>
       </c>
@@ -2410,7 +2413,7 @@
       </c>
       <c r="S4" s="6"/>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>406</v>
       </c>
@@ -2462,7 +2465,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>406</v>
       </c>
@@ -2507,7 +2510,7 @@
       </c>
       <c r="S6" s="6"/>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>406</v>
       </c>
@@ -2552,7 +2555,7 @@
       </c>
       <c r="S7" s="6"/>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>406</v>
       </c>
@@ -2599,7 +2602,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>406</v>
       </c>
@@ -2648,7 +2651,7 @@
       </c>
       <c r="S9" s="11"/>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>405</v>
       </c>
@@ -2697,7 +2700,7 @@
       </c>
       <c r="S10" s="11"/>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>162</v>
       </c>
@@ -2749,7 +2752,7 @@
       </c>
       <c r="S11" s="6"/>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>403</v>
       </c>
@@ -2794,7 +2797,7 @@
       </c>
       <c r="S12" s="6"/>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>403</v>
       </c>
@@ -2839,7 +2842,7 @@
       </c>
       <c r="S13" s="6"/>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>403</v>
       </c>
@@ -2886,7 +2889,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>403</v>
       </c>
@@ -2931,7 +2934,7 @@
       </c>
       <c r="S15" s="6"/>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>403</v>
       </c>
@@ -2976,7 +2979,7 @@
       </c>
       <c r="S16" s="6"/>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>403</v>
       </c>
@@ -3023,7 +3026,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>402</v>
       </c>
@@ -3068,7 +3071,7 @@
       </c>
       <c r="S18" s="6"/>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>401</v>
       </c>
@@ -3119,7 +3122,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>400</v>
       </c>
@@ -3164,7 +3167,7 @@
       </c>
       <c r="S20" s="6"/>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>399</v>
       </c>
@@ -3209,7 +3212,7 @@
       </c>
       <c r="S21" s="6"/>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>398</v>
       </c>
@@ -3254,7 +3257,7 @@
       </c>
       <c r="S22" s="6"/>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>398</v>
       </c>
@@ -3299,7 +3302,7 @@
       </c>
       <c r="S23" s="6"/>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>398</v>
       </c>
@@ -3346,7 +3349,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>393</v>
       </c>
@@ -3391,7 +3394,7 @@
       </c>
       <c r="S25" s="6"/>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>392</v>
       </c>
@@ -3436,7 +3439,7 @@
       </c>
       <c r="S26" s="6"/>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>392</v>
       </c>
@@ -3481,7 +3484,7 @@
       </c>
       <c r="S27" s="6"/>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>276</v>
       </c>
@@ -3528,7 +3531,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>419</v>
       </c>
@@ -3573,7 +3576,7 @@
       </c>
       <c r="S29" s="11"/>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>391</v>
       </c>
@@ -3618,7 +3621,7 @@
       </c>
       <c r="S30" s="6"/>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>389</v>
       </c>
@@ -3667,7 +3670,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>390</v>
       </c>
@@ -3714,7 +3717,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>387</v>
       </c>
@@ -3761,7 +3764,7 @@
       </c>
       <c r="S33" s="6"/>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>380</v>
       </c>
@@ -3815,7 +3818,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>379</v>
       </c>
@@ -3867,7 +3870,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>103</v>
       </c>
@@ -3919,7 +3922,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>347</v>
       </c>
@@ -3971,7 +3974,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>103</v>
       </c>
@@ -4018,7 +4021,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>103</v>
       </c>
@@ -4068,7 +4071,7 @@
       </c>
       <c r="S39" s="6"/>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>103</v>
       </c>
@@ -4117,7 +4120,7 @@
       </c>
       <c r="S40" s="11"/>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
         <v>103</v>
       </c>
@@ -4166,7 +4169,7 @@
       </c>
       <c r="S41" s="11"/>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
         <v>103</v>
       </c>
@@ -4216,7 +4219,7 @@
       </c>
       <c r="S42" s="11"/>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>103</v>
       </c>
@@ -4261,7 +4264,7 @@
       </c>
       <c r="S43" s="6"/>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>375</v>
       </c>
@@ -4306,7 +4309,7 @@
       </c>
       <c r="S44" s="6"/>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>375</v>
       </c>
@@ -4351,7 +4354,7 @@
       </c>
       <c r="S45" s="6"/>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>347</v>
       </c>
@@ -4401,7 +4404,7 @@
       </c>
       <c r="S46" s="6"/>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>351</v>
       </c>
@@ -4448,7 +4451,7 @@
       </c>
       <c r="S47" s="6"/>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>351</v>
       </c>
@@ -4495,7 +4498,7 @@
       </c>
       <c r="S48" s="6"/>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>356</v>
       </c>
@@ -4542,7 +4545,7 @@
       </c>
       <c r="S49" s="6"/>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>356</v>
       </c>
@@ -4594,7 +4597,7 @@
       </c>
       <c r="S50" s="6"/>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>356</v>
       </c>
@@ -4641,7 +4644,7 @@
       </c>
       <c r="S51" s="13"/>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>356</v>
       </c>
@@ -4693,7 +4696,7 @@
       </c>
       <c r="S52" s="6"/>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>356</v>
       </c>
@@ -4740,7 +4743,7 @@
       </c>
       <c r="S53" s="13"/>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>358</v>
       </c>
@@ -4787,7 +4790,7 @@
       </c>
       <c r="S54" s="6"/>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A55" s="13" t="s">
         <v>360</v>
       </c>
@@ -4836,7 +4839,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="13" t="s">
         <v>360</v>
       </c>
@@ -4883,7 +4886,7 @@
       </c>
       <c r="S56" s="13"/>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A57" s="13" t="s">
         <v>362</v>
       </c>
@@ -4930,7 +4933,7 @@
       </c>
       <c r="S57" s="13"/>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A58" s="13" t="s">
         <v>362</v>
       </c>
@@ -4977,7 +4980,7 @@
       </c>
       <c r="S58" s="13"/>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A59" s="13" t="s">
         <v>364</v>
       </c>
@@ -5024,7 +5027,7 @@
       </c>
       <c r="S59" s="13"/>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A60" s="13" t="s">
         <v>365</v>
       </c>
@@ -5076,7 +5079,7 @@
       </c>
       <c r="S60" s="13"/>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A61" s="13" t="s">
         <v>369</v>
       </c>
@@ -5123,7 +5126,7 @@
       </c>
       <c r="S61" s="13"/>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A62" s="13" t="s">
         <v>370</v>
       </c>
@@ -5170,7 +5173,7 @@
       </c>
       <c r="S62" s="13"/>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
         <v>371</v>
       </c>
@@ -5224,7 +5227,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
         <v>373</v>
       </c>
@@ -5273,7 +5276,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="65" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="65" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>356</v>
       </c>
@@ -5327,7 +5330,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="66" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="66" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>53</v>
       </c>
@@ -5379,7 +5382,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="67" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="67" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>330</v>
       </c>
@@ -5426,7 +5429,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="68" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="68" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>346</v>
       </c>
@@ -5471,7 +5474,7 @@
       </c>
       <c r="S68" s="6"/>
     </row>
-    <row r="69" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="69" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>145</v>
       </c>
@@ -5525,7 +5528,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="70" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="70" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>339</v>
       </c>
@@ -5572,7 +5575,7 @@
       </c>
       <c r="S70" s="6"/>
     </row>
-    <row r="71" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="71" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>339</v>
       </c>
@@ -5619,7 +5622,7 @@
       </c>
       <c r="S71" s="6"/>
     </row>
-    <row r="72" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="72" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>339</v>
       </c>
@@ -5666,7 +5669,7 @@
       </c>
       <c r="S72" s="6"/>
     </row>
-    <row r="73" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="73" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>339</v>
       </c>
@@ -5716,7 +5719,7 @@
       </c>
       <c r="S73" s="6"/>
     </row>
-    <row r="74" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="74" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>339</v>
       </c>
@@ -5765,7 +5768,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="75" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="75" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>342</v>
       </c>
@@ -5810,7 +5813,7 @@
       </c>
       <c r="S75" s="6"/>
     </row>
-    <row r="76" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="76" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>342</v>
       </c>
@@ -5857,7 +5860,7 @@
       </c>
       <c r="S76" s="6"/>
     </row>
-    <row r="77" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="77" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
         <v>344</v>
       </c>
@@ -5904,7 +5907,7 @@
       </c>
       <c r="S77" s="6"/>
     </row>
-    <row r="78" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="78" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>344</v>
       </c>
@@ -5953,7 +5956,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="79" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="79" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>345</v>
       </c>
@@ -5998,7 +6001,7 @@
       </c>
       <c r="S79" s="6"/>
     </row>
-    <row r="80" spans="1:27" x14ac:dyDescent="0.5">
+    <row r="80" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>414</v>
       </c>
@@ -6048,7 +6051,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A81" s="13" t="s">
         <v>336</v>
       </c>
@@ -6095,7 +6098,7 @@
       </c>
       <c r="S81" s="13"/>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
         <v>335</v>
       </c>
@@ -6140,7 +6143,7 @@
       </c>
       <c r="S82" s="6"/>
     </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A83" s="6" t="s">
         <v>327</v>
       </c>
@@ -6187,7 +6190,7 @@
       </c>
       <c r="S83" s="6"/>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A84" s="6" t="s">
         <v>321</v>
       </c>
@@ -6234,7 +6237,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
         <v>321</v>
       </c>
@@ -6281,7 +6284,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A86" s="6" t="s">
         <v>324</v>
       </c>
@@ -6328,7 +6331,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A87" s="11" t="s">
         <v>106</v>
       </c>
@@ -6378,7 +6381,7 @@
       </c>
       <c r="S87" s="6"/>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
         <v>320</v>
       </c>
@@ -6430,7 +6433,7 @@
       </c>
       <c r="S88" s="6"/>
     </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A89" s="6" t="s">
         <v>320</v>
       </c>
@@ -6482,7 +6485,7 @@
       </c>
       <c r="S89" s="6"/>
     </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A90" s="6" t="s">
         <v>320</v>
       </c>
@@ -6534,7 +6537,7 @@
       </c>
       <c r="S90" s="6"/>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A91" s="6" t="s">
         <v>385</v>
       </c>
@@ -6581,7 +6584,7 @@
       </c>
       <c r="S91" s="6"/>
     </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A92" s="13" t="s">
         <v>96</v>
       </c>
@@ -6633,7 +6636,7 @@
       </c>
       <c r="S92" s="13"/>
     </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A93" s="6" t="s">
         <v>316</v>
       </c>
@@ -6678,7 +6681,7 @@
       </c>
       <c r="S93" s="13"/>
     </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A94" s="6" t="s">
         <v>315</v>
       </c>
@@ -6723,7 +6726,7 @@
       </c>
       <c r="S94" s="6"/>
     </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A95" s="6" t="s">
         <v>315</v>
       </c>
@@ -6768,7 +6771,7 @@
       </c>
       <c r="S95" s="6"/>
     </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A96" s="6" t="s">
         <v>315</v>
       </c>
@@ -6813,7 +6816,7 @@
       </c>
       <c r="S96" s="6"/>
     </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="97" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A97" s="6" t="s">
         <v>311</v>
       </c>
@@ -6860,7 +6863,7 @@
       </c>
       <c r="S97" s="6"/>
     </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="98" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A98" s="6" t="s">
         <v>310</v>
       </c>
@@ -6911,7 +6914,7 @@
       </c>
       <c r="S98" s="6"/>
     </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="99" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A99" s="13" t="s">
         <v>308</v>
       </c>
@@ -6958,7 +6961,7 @@
       </c>
       <c r="S99" s="13"/>
     </row>
-    <row r="100" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="100" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A100" s="6" t="s">
         <v>304</v>
       </c>
@@ -7005,7 +7008,7 @@
       </c>
       <c r="S100" s="6"/>
     </row>
-    <row r="101" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="101" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
         <v>303</v>
       </c>
@@ -7050,7 +7053,7 @@
       </c>
       <c r="S101" s="13"/>
     </row>
-    <row r="102" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="102" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A102" s="6" t="s">
         <v>111</v>
       </c>
@@ -7102,7 +7105,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="103" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="103" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A103" s="6" t="s">
         <v>111</v>
       </c>
@@ -7149,7 +7152,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="104" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="104" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A104" s="6" t="s">
         <v>111</v>
       </c>
@@ -7194,7 +7197,7 @@
       </c>
       <c r="S104" s="6"/>
     </row>
-    <row r="105" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="105" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A105" s="6" t="s">
         <v>111</v>
       </c>
@@ -7239,7 +7242,7 @@
       </c>
       <c r="S105" s="6"/>
     </row>
-    <row r="106" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="106" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A106" s="6" t="s">
         <v>111</v>
       </c>
@@ -7284,7 +7287,7 @@
       </c>
       <c r="S106" s="6"/>
     </row>
-    <row r="107" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="107" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A107" s="6" t="s">
         <v>111</v>
       </c>
@@ -7331,7 +7334,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="108" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="108" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A108" s="6" t="s">
         <v>298</v>
       </c>
@@ -7383,7 +7386,7 @@
       </c>
       <c r="S108" s="6"/>
     </row>
-    <row r="109" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="109" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A109" s="6" t="s">
         <v>290</v>
       </c>
@@ -7433,7 +7436,7 @@
       </c>
       <c r="S109" s="6"/>
     </row>
-    <row r="110" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="110" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A110" s="6" t="s">
         <v>173</v>
       </c>
@@ -7485,7 +7488,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="111" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="111" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="11" t="s">
         <v>87</v>
       </c>
@@ -7537,7 +7540,7 @@
       </c>
       <c r="S111" s="11"/>
     </row>
-    <row r="112" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="112" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="11" t="s">
         <v>87</v>
       </c>
@@ -7584,7 +7587,7 @@
       </c>
       <c r="S112" s="11"/>
     </row>
-    <row r="113" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="113" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="11" t="s">
         <v>294</v>
       </c>
@@ -7631,7 +7634,7 @@
       </c>
       <c r="S113" s="6"/>
     </row>
-    <row r="114" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="114" spans="1:22" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="6" t="s">
         <v>289</v>
       </c>
@@ -7676,7 +7679,7 @@
       </c>
       <c r="S114" s="6"/>
     </row>
-    <row r="115" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="115" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A115" s="6" t="s">
         <v>287</v>
       </c>
@@ -7723,7 +7726,7 @@
       </c>
       <c r="S115" s="6"/>
     </row>
-    <row r="116" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="116" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A116" s="6" t="s">
         <v>142</v>
       </c>
@@ -7775,7 +7778,7 @@
       </c>
       <c r="S116" s="6"/>
     </row>
-    <row r="117" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="117" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A117" s="6" t="s">
         <v>283</v>
       </c>
@@ -7824,7 +7827,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="118" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="118" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A118" s="6" t="s">
         <v>145</v>
       </c>
@@ -7871,7 +7874,7 @@
       </c>
       <c r="S118" s="6"/>
     </row>
-    <row r="119" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="119" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A119" s="6" t="s">
         <v>285</v>
       </c>
@@ -7923,7 +7926,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="120" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="120" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A120" s="6" t="s">
         <v>285</v>
       </c>
@@ -7973,7 +7976,7 @@
       </c>
       <c r="S120" s="6"/>
     </row>
-    <row r="121" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="121" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A121" s="6" t="s">
         <v>285</v>
       </c>
@@ -8023,7 +8026,7 @@
       </c>
       <c r="S121" s="6"/>
     </row>
-    <row r="122" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="122" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A122" s="6" t="s">
         <v>173</v>
       </c>
@@ -8075,7 +8078,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="123" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="123" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A123" s="6" t="s">
         <v>173</v>
       </c>
@@ -8127,7 +8130,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="124" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="124" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A124" s="6" t="s">
         <v>173</v>
       </c>
@@ -8177,7 +8180,7 @@
       </c>
       <c r="S124" s="6"/>
     </row>
-    <row r="125" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="125" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A125" s="6" t="s">
         <v>276</v>
       </c>
@@ -8226,7 +8229,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="126" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="126" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A126" s="6" t="s">
         <v>53</v>
       </c>
@@ -8271,7 +8274,7 @@
       </c>
       <c r="S126" s="6"/>
     </row>
-    <row r="127" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="127" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A127" s="6" t="s">
         <v>53</v>
       </c>
@@ -8321,7 +8324,7 @@
       <c r="U127" s="3"/>
       <c r="V127" s="3"/>
     </row>
-    <row r="128" spans="1:22" x14ac:dyDescent="0.5">
+    <row r="128" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A128" s="11" t="s">
         <v>42</v>
       </c>
@@ -8366,7 +8369,7 @@
       </c>
       <c r="S128" s="6"/>
     </row>
-    <row r="129" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="129" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A129" s="6" t="s">
         <v>272</v>
       </c>
@@ -8413,7 +8416,7 @@
       </c>
       <c r="S129" s="6"/>
     </row>
-    <row r="130" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="130" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A130" s="6" t="s">
         <v>103</v>
       </c>
@@ -8463,7 +8466,7 @@
       </c>
       <c r="S130" s="6"/>
     </row>
-    <row r="131" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="131" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A131" s="13" t="s">
         <v>269</v>
       </c>
@@ -8511,7 +8514,7 @@
       <c r="S131" s="13"/>
       <c r="T131" s="3"/>
     </row>
-    <row r="132" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="132" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A132" s="13" t="s">
         <v>269</v>
       </c>
@@ -8565,7 +8568,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="133" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="133" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A133" s="6" t="s">
         <v>418</v>
       </c>
@@ -8610,7 +8613,7 @@
       </c>
       <c r="S133" s="6"/>
     </row>
-    <row r="134" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="134" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A134" s="6" t="s">
         <v>261</v>
       </c>
@@ -8655,7 +8658,7 @@
       </c>
       <c r="S134" s="6"/>
     </row>
-    <row r="135" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="135" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A135" s="6" t="s">
         <v>262</v>
       </c>
@@ -8705,7 +8708,7 @@
       </c>
       <c r="S135" s="6"/>
     </row>
-    <row r="136" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="136" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A136" s="6" t="s">
         <v>262</v>
       </c>
@@ -8757,7 +8760,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="137" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="137" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A137" s="6" t="s">
         <v>265</v>
       </c>
@@ -8802,7 +8805,7 @@
       </c>
       <c r="S137" s="6"/>
     </row>
-    <row r="138" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="138" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A138" s="6" t="s">
         <v>266</v>
       </c>
@@ -8847,7 +8850,7 @@
       </c>
       <c r="S138" s="6"/>
     </row>
-    <row r="139" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="139" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A139" s="6" t="s">
         <v>267</v>
       </c>
@@ -8892,7 +8895,7 @@
       </c>
       <c r="S139" s="6"/>
     </row>
-    <row r="140" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="140" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A140" s="6" t="s">
         <v>268</v>
       </c>
@@ -8937,7 +8940,7 @@
       </c>
       <c r="S140" s="6"/>
     </row>
-    <row r="141" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="141" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A141" s="6" t="s">
         <v>92</v>
       </c>
@@ -8989,7 +8992,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="142" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="142" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A142" s="6" t="s">
         <v>259</v>
       </c>
@@ -9036,7 +9039,7 @@
       </c>
       <c r="S142" s="13"/>
     </row>
-    <row r="143" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="143" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A143" s="6" t="s">
         <v>115</v>
       </c>
@@ -9081,7 +9084,7 @@
       </c>
       <c r="S143" s="6"/>
     </row>
-    <row r="144" spans="1:20" x14ac:dyDescent="0.5">
+    <row r="144" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A144" s="6" t="s">
         <v>257</v>
       </c>
@@ -9133,7 +9136,7 @@
       </c>
       <c r="S144" s="6"/>
     </row>
-    <row r="145" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="145" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A145" s="11" t="s">
         <v>252</v>
       </c>
@@ -9180,7 +9183,7 @@
       </c>
       <c r="S145" s="6"/>
     </row>
-    <row r="146" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="146" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A146" s="11" t="s">
         <v>252</v>
       </c>
@@ -9230,7 +9233,7 @@
       </c>
       <c r="S146" s="6"/>
     </row>
-    <row r="147" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="147" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A147" s="6" t="s">
         <v>227</v>
       </c>
@@ -9277,7 +9280,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="148" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="148" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A148" s="6" t="s">
         <v>227</v>
       </c>
@@ -9322,7 +9325,7 @@
       </c>
       <c r="S148" s="6"/>
     </row>
-    <row r="149" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="149" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A149" s="13" t="s">
         <v>228</v>
       </c>
@@ -9369,7 +9372,7 @@
       </c>
       <c r="S149" s="13"/>
     </row>
-    <row r="150" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="150" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A150" s="6" t="s">
         <v>108</v>
       </c>
@@ -9421,7 +9424,7 @@
       </c>
       <c r="S150" s="6"/>
     </row>
-    <row r="151" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="151" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A151" s="6" t="s">
         <v>108</v>
       </c>
@@ -9473,7 +9476,7 @@
       </c>
       <c r="S151" s="6"/>
     </row>
-    <row r="152" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="152" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A152" s="6" t="s">
         <v>225</v>
       </c>
@@ -9520,7 +9523,7 @@
       </c>
       <c r="S152" s="6"/>
     </row>
-    <row r="153" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="153" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A153" s="6" t="s">
         <v>213</v>
       </c>
@@ -9572,7 +9575,7 @@
       </c>
       <c r="S153" s="6"/>
     </row>
-    <row r="154" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="154" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A154" s="6" t="s">
         <v>108</v>
       </c>
@@ -9621,7 +9624,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="155" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="155" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A155" s="6" t="s">
         <v>218</v>
       </c>
@@ -9673,7 +9676,7 @@
       </c>
       <c r="S155" s="6"/>
     </row>
-    <row r="156" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="156" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A156" s="6" t="s">
         <v>218</v>
       </c>
@@ -9720,7 +9723,7 @@
       </c>
       <c r="S156" s="6"/>
     </row>
-    <row r="157" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="157" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A157" s="6" t="s">
         <v>223</v>
       </c>
@@ -9770,7 +9773,7 @@
       </c>
       <c r="S157" s="6"/>
     </row>
-    <row r="158" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="158" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A158" s="6" t="s">
         <v>223</v>
       </c>
@@ -9817,7 +9820,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="159" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="159" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A159" s="6" t="s">
         <v>223</v>
       </c>
@@ -9862,7 +9865,7 @@
       </c>
       <c r="S159" s="6"/>
     </row>
-    <row r="160" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="160" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A160" s="6" t="s">
         <v>223</v>
       </c>
@@ -9909,7 +9912,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="161" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="161" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A161" s="6" t="s">
         <v>223</v>
       </c>
@@ -9954,7 +9957,7 @@
       </c>
       <c r="S161" s="6"/>
     </row>
-    <row r="162" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="162" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A162" s="6" t="s">
         <v>223</v>
       </c>
@@ -9999,7 +10002,7 @@
       </c>
       <c r="S162" s="6"/>
     </row>
-    <row r="163" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="163" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A163" s="6" t="s">
         <v>223</v>
       </c>
@@ -10044,7 +10047,7 @@
       </c>
       <c r="S163" s="6"/>
     </row>
-    <row r="164" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="164" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A164" s="6" t="s">
         <v>223</v>
       </c>
@@ -10089,7 +10092,7 @@
       </c>
       <c r="S164" s="6"/>
     </row>
-    <row r="165" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="165" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A165" s="6" t="s">
         <v>115</v>
       </c>
@@ -10141,7 +10144,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="166" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="166" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A166" s="6" t="s">
         <v>111</v>
       </c>
@@ -10188,7 +10191,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="167" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="167" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A167" s="6" t="s">
         <v>211</v>
       </c>
@@ -10233,7 +10236,7 @@
       </c>
       <c r="S167" s="6"/>
     </row>
-    <row r="168" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="168" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A168" s="6" t="s">
         <v>211</v>
       </c>
@@ -10280,7 +10283,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="169" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="169" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A169" s="6" t="s">
         <v>211</v>
       </c>
@@ -10325,7 +10328,7 @@
       </c>
       <c r="S169" s="6"/>
     </row>
-    <row r="170" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="170" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A170" s="11" t="s">
         <v>212</v>
       </c>
@@ -10377,7 +10380,7 @@
       </c>
       <c r="S170" s="6"/>
     </row>
-    <row r="171" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="171" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A171" s="11" t="s">
         <v>338</v>
       </c>
@@ -10431,7 +10434,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="172" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="172" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A172" s="6" t="s">
         <v>209</v>
       </c>
@@ -10485,7 +10488,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="173" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="173" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A173" s="6" t="s">
         <v>209</v>
       </c>
@@ -10532,7 +10535,7 @@
       </c>
       <c r="S173" s="6"/>
     </row>
-    <row r="174" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="174" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A174" s="6" t="s">
         <v>209</v>
       </c>
@@ -10579,7 +10582,7 @@
       </c>
       <c r="S174" s="6"/>
     </row>
-    <row r="175" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="175" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A175" s="6" t="s">
         <v>209</v>
       </c>
@@ -10626,7 +10629,7 @@
       </c>
       <c r="S175" s="6"/>
     </row>
-    <row r="176" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="176" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A176" s="6" t="s">
         <v>145</v>
       </c>
@@ -10673,7 +10676,7 @@
       </c>
       <c r="S176" s="6"/>
     </row>
-    <row r="177" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="177" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A177" s="11" t="s">
         <v>186</v>
       </c>
@@ -10720,7 +10723,7 @@
       </c>
       <c r="S177" s="6"/>
     </row>
-    <row r="178" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="178" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A178" s="11" t="s">
         <v>188</v>
       </c>
@@ -10770,7 +10773,7 @@
       </c>
       <c r="S178" s="6"/>
     </row>
-    <row r="179" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="179" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A179" s="13" t="s">
         <v>170</v>
       </c>
@@ -10817,7 +10820,7 @@
       </c>
       <c r="S179" s="13"/>
     </row>
-    <row r="180" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="180" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A180" s="13" t="s">
         <v>170</v>
       </c>
@@ -10864,7 +10867,7 @@
       </c>
       <c r="S180" s="13"/>
     </row>
-    <row r="181" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="181" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A181" s="13" t="s">
         <v>170</v>
       </c>
@@ -10913,7 +10916,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="182" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="182" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A182" s="13" t="s">
         <v>184</v>
       </c>
@@ -10960,7 +10963,7 @@
       </c>
       <c r="S182" s="13"/>
     </row>
-    <row r="183" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="183" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A183" s="13" t="s">
         <v>170</v>
       </c>
@@ -11014,7 +11017,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="184" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="184" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A184" s="6" t="s">
         <v>162</v>
       </c>
@@ -11061,7 +11064,7 @@
       </c>
       <c r="S184" s="6"/>
     </row>
-    <row r="185" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="185" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A185" s="6" t="s">
         <v>164</v>
       </c>
@@ -11108,7 +11111,7 @@
       </c>
       <c r="S185" s="6"/>
     </row>
-    <row r="186" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="186" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A186" s="6" t="s">
         <v>165</v>
       </c>
@@ -11160,7 +11163,7 @@
       </c>
       <c r="S186" s="6"/>
     </row>
-    <row r="187" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="187" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A187" s="6" t="s">
         <v>160</v>
       </c>
@@ -11214,7 +11217,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="188" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="188" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A188" s="11" t="s">
         <v>110</v>
       </c>
@@ -11264,7 +11267,7 @@
       </c>
       <c r="S188" s="6"/>
     </row>
-    <row r="189" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="189" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A189" s="6" t="s">
         <v>139</v>
       </c>
@@ -11311,7 +11314,7 @@
       </c>
       <c r="S189" s="6"/>
     </row>
-    <row r="190" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="190" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A190" s="6" t="s">
         <v>139</v>
       </c>
@@ -11360,7 +11363,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="191" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="191" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A191" s="6" t="s">
         <v>139</v>
       </c>
@@ -11409,7 +11412,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="192" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="192" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A192" s="6" t="s">
         <v>138</v>
       </c>
@@ -11456,7 +11459,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="193" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="193" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A193" s="6" t="s">
         <v>138</v>
       </c>
@@ -11501,7 +11504,7 @@
       </c>
       <c r="S193" s="6"/>
     </row>
-    <row r="194" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="194" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A194" s="11" t="s">
         <v>87</v>
       </c>
@@ -11548,7 +11551,7 @@
       </c>
       <c r="S194" s="11"/>
     </row>
-    <row r="195" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="195" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A195" s="11" t="s">
         <v>137</v>
       </c>
@@ -11595,7 +11598,7 @@
       </c>
       <c r="S195" s="6"/>
     </row>
-    <row r="196" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="196" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A196" s="11" t="s">
         <v>87</v>
       </c>
@@ -11642,7 +11645,7 @@
       </c>
       <c r="S196" s="11"/>
     </row>
-    <row r="197" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="197" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A197" s="11" t="s">
         <v>116</v>
       </c>
@@ -11694,7 +11697,7 @@
       </c>
       <c r="S197" s="6"/>
     </row>
-    <row r="198" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="198" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A198" s="11" t="s">
         <v>116</v>
       </c>
@@ -11748,7 +11751,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="199" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="199" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A199" s="11" t="s">
         <v>173</v>
       </c>
@@ -11802,7 +11805,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="200" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="200" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A200" s="11" t="s">
         <v>226</v>
       </c>
@@ -11854,7 +11857,7 @@
       </c>
       <c r="S200" s="6"/>
     </row>
-    <row r="201" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="201" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A201" s="11" t="s">
         <v>226</v>
       </c>
@@ -11906,7 +11909,7 @@
       </c>
       <c r="S201" s="6"/>
     </row>
-    <row r="202" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="202" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A202" s="11" t="s">
         <v>226</v>
       </c>
@@ -11960,7 +11963,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="203" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="203" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A203" s="11" t="s">
         <v>226</v>
       </c>
@@ -12012,7 +12015,7 @@
       </c>
       <c r="S203" s="6"/>
     </row>
-    <row r="204" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="204" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A204" s="11" t="s">
         <v>226</v>
       </c>
@@ -12064,7 +12067,7 @@
       </c>
       <c r="S204" s="6"/>
     </row>
-    <row r="205" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="205" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A205" s="11" t="s">
         <v>226</v>
       </c>
@@ -12116,7 +12119,7 @@
       </c>
       <c r="S205" s="6"/>
     </row>
-    <row r="206" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="206" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A206" s="11" t="s">
         <v>226</v>
       </c>
@@ -12168,7 +12171,7 @@
       </c>
       <c r="S206" s="6"/>
     </row>
-    <row r="207" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="207" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A207" s="11" t="s">
         <v>119</v>
       </c>
@@ -12215,7 +12218,7 @@
       </c>
       <c r="S207" s="6"/>
     </row>
-    <row r="208" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="208" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A208" s="11" t="s">
         <v>135</v>
       </c>
@@ -12262,7 +12265,7 @@
       </c>
       <c r="S208" s="6"/>
     </row>
-    <row r="209" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="209" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A209" s="6" t="s">
         <v>111</v>
       </c>
@@ -12309,7 +12312,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="210" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="210" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A210" s="6" t="s">
         <v>111</v>
       </c>
@@ -12356,7 +12359,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="211" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="211" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A211" s="6" t="s">
         <v>111</v>
       </c>
@@ -12403,7 +12406,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="212" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="212" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A212" s="6" t="s">
         <v>111</v>
       </c>
@@ -12448,7 +12451,7 @@
       </c>
       <c r="S212" s="6"/>
     </row>
-    <row r="213" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="213" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A213" s="6" t="s">
         <v>111</v>
       </c>
@@ -12493,7 +12496,7 @@
       </c>
       <c r="S213" s="6"/>
     </row>
-    <row r="214" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="214" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A214" s="6" t="s">
         <v>326</v>
       </c>
@@ -12547,7 +12550,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="215" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="215" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A215" s="6" t="s">
         <v>352</v>
       </c>
@@ -12594,7 +12597,7 @@
       </c>
       <c r="S215" s="13"/>
     </row>
-    <row r="216" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="216" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A216" s="6" t="s">
         <v>353</v>
       </c>
@@ -12641,7 +12644,7 @@
       </c>
       <c r="S216" s="13"/>
     </row>
-    <row r="217" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="217" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A217" s="6" t="s">
         <v>353</v>
       </c>
@@ -12688,7 +12691,7 @@
       </c>
       <c r="S217" s="13"/>
     </row>
-    <row r="218" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="218" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A218" s="6" t="s">
         <v>353</v>
       </c>
@@ -12737,7 +12740,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="219" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="219" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A219" s="6" t="s">
         <v>20</v>
       </c>
@@ -12782,7 +12785,7 @@
       </c>
       <c r="S219" s="6"/>
     </row>
-    <row r="220" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="220" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A220" s="6" t="s">
         <v>220</v>
       </c>
@@ -12827,7 +12830,7 @@
       </c>
       <c r="S220" s="6"/>
     </row>
-    <row r="221" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="221" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A221" s="6" t="s">
         <v>220</v>
       </c>
@@ -12872,7 +12875,7 @@
       </c>
       <c r="S221" s="6"/>
     </row>
-    <row r="222" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="222" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A222" s="6" t="s">
         <v>220</v>
       </c>
@@ -12917,7 +12920,7 @@
       </c>
       <c r="S222" s="6"/>
     </row>
-    <row r="223" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="223" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A223" s="6" t="s">
         <v>220</v>
       </c>
@@ -12962,7 +12965,7 @@
       </c>
       <c r="S223" s="6"/>
     </row>
-    <row r="224" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="224" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A224" s="6" t="s">
         <v>220</v>
       </c>
@@ -13009,7 +13012,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="225" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="225" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A225" s="6" t="s">
         <v>220</v>
       </c>
@@ -13054,7 +13057,7 @@
       </c>
       <c r="S225" s="6"/>
     </row>
-    <row r="226" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="226" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A226" s="11" t="s">
         <v>100</v>
       </c>
@@ -13101,7 +13104,7 @@
       </c>
       <c r="S226" s="6"/>
     </row>
-    <row r="227" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="227" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A227" s="6" t="s">
         <v>354</v>
       </c>
@@ -13148,7 +13151,7 @@
       </c>
       <c r="S227" s="13"/>
     </row>
-    <row r="228" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="228" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A228" s="11" t="s">
         <v>189</v>
       </c>
@@ -13195,7 +13198,7 @@
       </c>
       <c r="S228" s="6"/>
     </row>
-    <row r="229" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="229" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A229" s="11" t="s">
         <v>133</v>
       </c>
@@ -13247,7 +13250,7 @@
       </c>
       <c r="S229" s="6"/>
     </row>
-    <row r="230" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="230" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A230" s="11" t="s">
         <v>318</v>
       </c>
@@ -13296,7 +13299,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="231" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="231" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A231" s="11" t="s">
         <v>318</v>
       </c>
@@ -13343,7 +13346,7 @@
       </c>
       <c r="S231" s="6"/>
     </row>
-    <row r="232" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="232" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A232" s="6" t="s">
         <v>330</v>
       </c>
@@ -13395,7 +13398,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="233" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="233" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A233" s="6" t="s">
         <v>213</v>
       </c>
@@ -13449,7 +13452,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="234" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="234" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A234" s="6" t="s">
         <v>83</v>
       </c>
@@ -13496,7 +13499,7 @@
       </c>
       <c r="S234" s="6"/>
     </row>
-    <row r="235" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="235" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A235" s="6" t="s">
         <v>83</v>
       </c>
@@ -13543,7 +13546,7 @@
       </c>
       <c r="S235" s="6"/>
     </row>
-    <row r="236" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="236" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A236" s="11" t="s">
         <v>121</v>
       </c>
@@ -13595,7 +13598,7 @@
       </c>
       <c r="S236" s="6"/>
     </row>
-    <row r="237" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="237" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A237" s="11" t="s">
         <v>121</v>
       </c>
@@ -13647,7 +13650,7 @@
       </c>
       <c r="S237" s="6"/>
     </row>
-    <row r="238" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="238" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A238" s="11" t="s">
         <v>121</v>
       </c>
@@ -13699,7 +13702,7 @@
       </c>
       <c r="S238" s="6"/>
     </row>
-    <row r="239" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="239" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A239" s="11" t="s">
         <v>129</v>
       </c>
@@ -13746,7 +13749,7 @@
       </c>
       <c r="S239" s="6"/>
     </row>
-    <row r="240" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="240" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A240" s="11" t="s">
         <v>129</v>
       </c>
@@ -13798,7 +13801,7 @@
       </c>
       <c r="S240" s="6"/>
     </row>
-    <row r="241" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="241" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A241" s="6" t="s">
         <v>148</v>
       </c>
@@ -13852,7 +13855,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="242" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="242" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A242" s="13" t="s">
         <v>180</v>
       </c>
@@ -13899,7 +13902,7 @@
       </c>
       <c r="S242" s="13"/>
     </row>
-    <row r="243" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="243" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A243" s="13" t="s">
         <v>182</v>
       </c>
@@ -13946,7 +13949,7 @@
       </c>
       <c r="S243" s="13"/>
     </row>
-    <row r="244" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="244" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A244" s="6" t="s">
         <v>328</v>
       </c>
@@ -13991,7 +13994,7 @@
       </c>
       <c r="S244" s="6"/>
     </row>
-    <row r="245" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="245" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A245" s="6" t="s">
         <v>328</v>
       </c>
@@ -14036,7 +14039,7 @@
       </c>
       <c r="S245" s="6"/>
     </row>
-    <row r="246" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="246" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A246" s="6" t="s">
         <v>328</v>
       </c>
@@ -14083,7 +14086,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="247" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="247" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A247" s="11" t="s">
         <v>355</v>
       </c>
@@ -14133,7 +14136,7 @@
       </c>
       <c r="S247" s="13"/>
     </row>
-    <row r="248" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="248" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A248" s="11" t="s">
         <v>192</v>
       </c>
@@ -14185,7 +14188,7 @@
       </c>
       <c r="S248" s="6"/>
     </row>
-    <row r="249" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="249" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A249" s="11" t="s">
         <v>193</v>
       </c>
@@ -14237,7 +14240,7 @@
       </c>
       <c r="S249" s="6"/>
     </row>
-    <row r="250" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="250" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A250" s="11" t="s">
         <v>256</v>
       </c>
@@ -14286,7 +14289,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="251" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="251" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A251" s="11" t="s">
         <v>157</v>
       </c>
@@ -14340,7 +14343,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="252" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="252" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A252" s="6" t="s">
         <v>330</v>
       </c>
@@ -14385,7 +14388,7 @@
       </c>
       <c r="S252" s="6"/>
     </row>
-    <row r="253" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="253" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A253" s="6" t="s">
         <v>381</v>
       </c>
@@ -14432,7 +14435,7 @@
       </c>
       <c r="S253" s="6"/>
     </row>
-    <row r="254" spans="1:19" s="49" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="254" spans="1:19" s="49" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A254" s="44" t="s">
         <v>254</v>
       </c>
@@ -14479,7 +14482,7 @@
       </c>
       <c r="S254" s="45"/>
     </row>
-    <row r="255" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="255" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A255" s="6" t="s">
         <v>382</v>
       </c>
@@ -14526,7 +14529,7 @@
       </c>
       <c r="S255" s="6"/>
     </row>
-    <row r="256" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="256" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A256" s="11" t="s">
         <v>125</v>
       </c>
@@ -14578,7 +14581,7 @@
       </c>
       <c r="S256" s="6"/>
     </row>
-    <row r="257" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="257" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A257" s="6" t="s">
         <v>208</v>
       </c>
@@ -14625,7 +14628,7 @@
       </c>
       <c r="S257" s="6"/>
     </row>
-    <row r="258" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="258" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A258" s="6" t="s">
         <v>395</v>
       </c>
@@ -14672,7 +14675,7 @@
       </c>
       <c r="S258" s="13"/>
     </row>
-    <row r="259" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="259" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A259" s="6" t="s">
         <v>397</v>
       </c>
@@ -14724,7 +14727,7 @@
       </c>
       <c r="S259" s="6"/>
     </row>
-    <row r="260" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="260" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A260" s="6" t="s">
         <v>384</v>
       </c>
@@ -14773,7 +14776,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="261" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="261" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A261" s="6" t="s">
         <v>198</v>
       </c>
@@ -14820,7 +14823,7 @@
       </c>
       <c r="S261" s="6"/>
     </row>
-    <row r="262" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="262" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A262" s="6" t="s">
         <v>335</v>
       </c>
@@ -14865,7 +14868,7 @@
       </c>
       <c r="S262" s="6"/>
     </row>
-    <row r="263" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="263" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A263" s="13" t="s">
         <v>367</v>
       </c>
@@ -14912,7 +14915,7 @@
       </c>
       <c r="S263" s="13"/>
     </row>
-    <row r="264" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="264" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A264" s="13" t="s">
         <v>368</v>
       </c>
@@ -14959,7 +14962,7 @@
       </c>
       <c r="S264" s="13"/>
     </row>
-    <row r="265" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="265" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A265" s="6" t="s">
         <v>394</v>
       </c>
@@ -15006,7 +15009,7 @@
       </c>
       <c r="S265" s="6"/>
     </row>
-    <row r="266" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="266" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A266" s="6" t="s">
         <v>80</v>
       </c>
@@ -15053,7 +15056,7 @@
       </c>
       <c r="S266" s="6"/>
     </row>
-    <row r="267" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="267" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A267" s="6" t="s">
         <v>145</v>
       </c>
@@ -15105,7 +15108,7 @@
       </c>
       <c r="S267" s="6"/>
     </row>
-    <row r="268" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="268" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A268" s="6" t="s">
         <v>145</v>
       </c>
@@ -15152,7 +15155,7 @@
       </c>
       <c r="S268" s="6"/>
     </row>
-    <row r="269" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="269" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A269" s="6" t="s">
         <v>145</v>
       </c>
@@ -15204,7 +15207,7 @@
       </c>
       <c r="S269" s="6"/>
     </row>
-    <row r="270" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="270" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A270" s="6" t="s">
         <v>53</v>
       </c>
@@ -15251,7 +15254,7 @@
       </c>
       <c r="S270" s="6"/>
     </row>
-    <row r="271" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="271" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A271" s="6" t="s">
         <v>63</v>
       </c>
@@ -15298,7 +15301,7 @@
       </c>
       <c r="S271" s="6"/>
     </row>
-    <row r="272" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="272" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A272" s="6" t="s">
         <v>63</v>
       </c>
@@ -15345,7 +15348,7 @@
       </c>
       <c r="S272" s="6"/>
     </row>
-    <row r="273" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="273" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A273" s="6" t="s">
         <v>63</v>
       </c>
@@ -15392,7 +15395,7 @@
       </c>
       <c r="S273" s="6"/>
     </row>
-    <row r="274" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="274" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A274" s="6" t="s">
         <v>63</v>
       </c>
@@ -15441,7 +15444,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="275" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="275" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A275" s="6" t="s">
         <v>63</v>
       </c>
@@ -15488,7 +15491,7 @@
       </c>
       <c r="S275" s="9"/>
     </row>
-    <row r="276" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="276" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A276" s="6" t="s">
         <v>63</v>
       </c>
@@ -15537,7 +15540,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="277" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="277" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A277" s="11" t="s">
         <v>128</v>
       </c>
@@ -15582,7 +15585,7 @@
       </c>
       <c r="S277" s="6"/>
     </row>
-    <row r="278" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="278" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A278" s="6" t="s">
         <v>57</v>
       </c>
@@ -15634,7 +15637,7 @@
       </c>
       <c r="S278" s="6"/>
     </row>
-    <row r="279" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="279" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A279" s="6" t="s">
         <v>145</v>
       </c>
@@ -15681,7 +15684,7 @@
       </c>
       <c r="S279" s="6"/>
     </row>
-    <row r="280" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="280" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A280" s="11" t="s">
         <v>194</v>
       </c>
@@ -15728,7 +15731,7 @@
       </c>
       <c r="S280" s="6"/>
     </row>
-    <row r="281" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="281" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A281" s="11" t="s">
         <v>195</v>
       </c>
@@ -15775,7 +15778,7 @@
       </c>
       <c r="S281" s="6"/>
     </row>
-    <row r="282" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="282" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A282" s="13" t="s">
         <v>234</v>
       </c>
@@ -15827,7 +15830,7 @@
       </c>
       <c r="S282" s="13"/>
     </row>
-    <row r="283" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="283" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A283" s="13" t="s">
         <v>234</v>
       </c>
@@ -15879,7 +15882,7 @@
       </c>
       <c r="S283" s="13"/>
     </row>
-    <row r="284" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="284" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A284" s="13" t="s">
         <v>234</v>
       </c>
@@ -15931,7 +15934,7 @@
       </c>
       <c r="S284" s="13"/>
     </row>
-    <row r="285" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="285" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A285" s="13" t="s">
         <v>234</v>
       </c>
@@ -15983,7 +15986,7 @@
       </c>
       <c r="S285" s="13"/>
     </row>
-    <row r="286" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="286" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A286" s="13" t="s">
         <v>234</v>
       </c>
@@ -16035,7 +16038,7 @@
       </c>
       <c r="S286" s="6"/>
     </row>
-    <row r="287" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="287" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A287" s="13" t="s">
         <v>244</v>
       </c>
@@ -16082,7 +16085,7 @@
       </c>
       <c r="S287" s="6"/>
     </row>
-    <row r="288" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="288" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A288" s="6" t="s">
         <v>334</v>
       </c>
@@ -16127,7 +16130,7 @@
       </c>
       <c r="S288" s="6"/>
     </row>
-    <row r="289" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="289" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A289" s="13" t="s">
         <v>237</v>
       </c>
@@ -16174,7 +16177,7 @@
       </c>
       <c r="S289" s="6"/>
     </row>
-    <row r="290" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="290" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A290" s="13" t="s">
         <v>249</v>
       </c>
@@ -16223,7 +16226,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="291" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="291" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A291" s="13" t="s">
         <v>251</v>
       </c>
@@ -16268,7 +16271,7 @@
       </c>
       <c r="S291" s="6"/>
     </row>
-    <row r="292" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="292" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A292" s="6" t="s">
         <v>333</v>
       </c>
@@ -16318,7 +16321,7 @@
       </c>
       <c r="S292" s="6"/>
     </row>
-    <row r="293" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="293" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A293" s="6" t="s">
         <v>333</v>
       </c>
@@ -16363,7 +16366,7 @@
       </c>
       <c r="S293" s="6"/>
     </row>
-    <row r="294" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="294" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A294" s="13" t="s">
         <v>177</v>
       </c>
@@ -16414,7 +16417,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="295" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="295" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A295" s="6" t="s">
         <v>204</v>
       </c>
@@ -16463,7 +16466,7 @@
       </c>
       <c r="S295" s="6"/>
     </row>
-    <row r="296" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="296" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A296" s="6" t="s">
         <v>204</v>
       </c>
@@ -16510,7 +16513,7 @@
       </c>
       <c r="S296" s="6"/>
     </row>
-    <row r="297" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="297" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A297" s="6" t="s">
         <v>206</v>
       </c>
@@ -16557,7 +16560,7 @@
       </c>
       <c r="S297" s="6"/>
     </row>
-    <row r="298" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="298" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A298" s="13" t="s">
         <v>248</v>
       </c>
@@ -16604,7 +16607,7 @@
       </c>
       <c r="S298" s="6"/>
     </row>
-    <row r="299" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="299" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A299" s="6" t="s">
         <v>331</v>
       </c>
@@ -16649,7 +16652,7 @@
       </c>
       <c r="S299" s="6"/>
     </row>
-    <row r="300" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="300" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A300" s="6" t="s">
         <v>331</v>
       </c>
@@ -16694,7 +16697,7 @@
       </c>
       <c r="S300" s="6"/>
     </row>
-    <row r="301" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="301" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A301" s="6" t="s">
         <v>331</v>
       </c>
@@ -16741,7 +16744,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="302" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="302" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A302" s="6" t="s">
         <v>332</v>
       </c>
@@ -16786,7 +16789,7 @@
       </c>
       <c r="S302" s="6"/>
     </row>
-    <row r="303" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="303" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A303" s="13" t="s">
         <v>239</v>
       </c>
@@ -16833,7 +16836,7 @@
       </c>
       <c r="S303" s="6"/>
     </row>
-    <row r="304" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="304" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A304" s="13" t="s">
         <v>241</v>
       </c>
@@ -16880,7 +16883,7 @@
       </c>
       <c r="S304" s="6"/>
     </row>
-    <row r="305" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="305" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A305" s="13" t="s">
         <v>246</v>
       </c>
@@ -16927,7 +16930,7 @@
       </c>
       <c r="S305" s="6"/>
     </row>
-    <row r="306" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="306" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A306" s="6" t="s">
         <v>143</v>
       </c>
@@ -16974,7 +16977,7 @@
       </c>
       <c r="S306" s="6"/>
     </row>
-    <row r="307" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="307" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A307" s="6" t="s">
         <v>200</v>
       </c>
@@ -17021,7 +17024,7 @@
       </c>
       <c r="S307" s="6"/>
     </row>
-    <row r="308" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="308" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A308" s="6" t="s">
         <v>201</v>
       </c>
@@ -17068,7 +17071,7 @@
       </c>
       <c r="S308" s="6"/>
     </row>
-    <row r="309" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="309" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A309" s="6" t="s">
         <v>202</v>
       </c>
@@ -17115,7 +17118,7 @@
       </c>
       <c r="S309" s="6"/>
     </row>
-    <row r="310" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="310" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A310" s="6" t="s">
         <v>388</v>
       </c>
@@ -17162,7 +17165,7 @@
       </c>
       <c r="S310" s="6"/>
     </row>
-    <row r="311" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="311" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A311" s="13" t="s">
         <v>36</v>
       </c>
@@ -17209,7 +17212,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="312" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="312" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A312" s="6" t="s">
         <v>348</v>
       </c>
@@ -17258,7 +17261,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="313" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="313" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A313" s="6" t="s">
         <v>348</v>
       </c>
@@ -17305,7 +17308,7 @@
       </c>
       <c r="S313" s="6"/>
     </row>
-    <row r="314" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="314" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A314" s="6" t="s">
         <v>348</v>
       </c>
@@ -17354,7 +17357,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="315" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="315" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A315" s="6" t="s">
         <v>313</v>
       </c>
@@ -17399,7 +17402,7 @@
       </c>
       <c r="S315" s="6"/>
     </row>
-    <row r="316" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="316" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A316" s="6" t="s">
         <v>407</v>
       </c>
@@ -17444,7 +17447,7 @@
       </c>
       <c r="S316" s="6"/>
     </row>
-    <row r="317" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="317" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A317" s="6" t="s">
         <v>409</v>
       </c>
@@ -17491,7 +17494,7 @@
       </c>
       <c r="S317" s="6"/>
     </row>
-    <row r="318" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="318" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A318" s="11" t="s">
         <v>411</v>
       </c>
@@ -17538,7 +17541,7 @@
       </c>
       <c r="S318" s="11"/>
     </row>
-    <row r="319" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="319" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A319" s="11" t="s">
         <v>411</v>
       </c>
@@ -17587,7 +17590,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="320" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="320" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A320" s="11" t="s">
         <v>412</v>
       </c>
@@ -17634,7 +17637,7 @@
       </c>
       <c r="S320" s="11"/>
     </row>
-    <row r="321" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="321" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A321" s="6" t="s">
         <v>292</v>
       </c>
@@ -17681,7 +17684,7 @@
       </c>
       <c r="S321" s="11"/>
     </row>
-    <row r="322" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="322" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A322" s="6" t="s">
         <v>413</v>
       </c>
@@ -17726,7 +17729,7 @@
       </c>
       <c r="S322" s="6"/>
     </row>
-    <row r="323" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="323" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A323" s="11" t="s">
         <v>421</v>
       </c>
@@ -17775,7 +17778,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="324" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="324" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A324" s="13" t="s">
         <v>313</v>
       </c>
@@ -17826,7 +17829,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="325" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="325" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A325" s="11" t="s">
         <v>306</v>
       </c>
@@ -17875,7 +17878,7 @@
       </c>
       <c r="S325" s="11"/>
     </row>
-    <row r="326" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="326" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A326" s="6" t="s">
         <v>337</v>
       </c>
@@ -17922,7 +17925,7 @@
       </c>
       <c r="S326" s="6"/>
     </row>
-    <row r="327" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="327" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A327" s="13" t="s">
         <v>306</v>
       </c>
@@ -17971,7 +17974,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="328" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="328" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A328" s="6" t="s">
         <v>297</v>
       </c>
@@ -18018,7 +18021,7 @@
       </c>
       <c r="S328" s="6"/>
     </row>
-    <row r="329" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="329" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A329" s="6" t="s">
         <v>317</v>
       </c>
@@ -18063,7 +18066,7 @@
       </c>
       <c r="S329" s="6"/>
     </row>
-    <row r="330" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="330" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A330" s="6" t="s">
         <v>313</v>
       </c>
@@ -18110,7 +18113,7 @@
       </c>
       <c r="S330" s="6"/>
     </row>
-    <row r="331" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="331" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A331" s="6" t="s">
         <v>292</v>
       </c>
@@ -18157,7 +18160,7 @@
       </c>
       <c r="S331" s="11"/>
     </row>
-    <row r="332" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="332" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A332" s="6" t="s">
         <v>306</v>
       </c>
@@ -18204,7 +18207,7 @@
       </c>
       <c r="S332" s="6"/>
     </row>
-    <row r="333" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="333" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A333" s="6" t="s">
         <v>307</v>
       </c>
@@ -18251,7 +18254,7 @@
       </c>
       <c r="S333" s="6"/>
     </row>
-    <row r="334" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="334" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A334" s="6" t="s">
         <v>297</v>
       </c>
@@ -18298,7 +18301,7 @@
       </c>
       <c r="S334" s="6"/>
     </row>
-    <row r="335" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="335" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A335" s="6" t="s">
         <v>297</v>
       </c>
@@ -18349,7 +18352,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="336" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="336" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A336" s="6" t="s">
         <v>292</v>
       </c>
@@ -18396,7 +18399,7 @@
       </c>
       <c r="S336" s="6"/>
     </row>
-    <row r="337" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="337" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A337" s="6" t="s">
         <v>296</v>
       </c>
@@ -18443,7 +18446,7 @@
       </c>
       <c r="S337" s="6"/>
     </row>
-    <row r="338" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="338" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A338" s="6" t="s">
         <v>297</v>
       </c>
@@ -18490,7 +18493,7 @@
       </c>
       <c r="S338" s="6"/>
     </row>
-    <row r="339" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="339" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A339" s="6" t="s">
         <v>281</v>
       </c>
@@ -18537,7 +18540,7 @@
       </c>
       <c r="S339" s="6"/>
     </row>
-    <row r="340" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="340" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A340" s="6" t="s">
         <v>277</v>
       </c>
@@ -18582,7 +18585,7 @@
       </c>
       <c r="S340" s="6"/>
     </row>
-    <row r="341" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="341" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A341" s="6" t="s">
         <v>278</v>
       </c>
@@ -18627,7 +18630,7 @@
       </c>
       <c r="S341" s="6"/>
     </row>
-    <row r="342" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="342" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A342" s="6" t="s">
         <v>279</v>
       </c>
@@ -18672,7 +18675,7 @@
       </c>
       <c r="S342" s="6"/>
     </row>
-    <row r="343" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="343" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A343" s="6" t="s">
         <v>280</v>
       </c>
@@ -18717,7 +18720,7 @@
       </c>
       <c r="S343" s="6"/>
     </row>
-    <row r="344" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="344" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A344" s="11" t="s">
         <v>275</v>
       </c>
@@ -18766,7 +18769,7 @@
       </c>
       <c r="S344" s="11"/>
     </row>
-    <row r="345" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="345" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A345" s="13" t="s">
         <v>229</v>
       </c>
@@ -18817,7 +18820,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="346" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="346" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A346" s="13" t="s">
         <v>229</v>
       </c>
@@ -18868,7 +18871,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="347" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="347" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A347" s="13" t="s">
         <v>229</v>
       </c>
@@ -18919,7 +18922,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="348" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="348" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A348" s="13" t="s">
         <v>229</v>
       </c>
@@ -18968,7 +18971,7 @@
       </c>
       <c r="S348" s="13"/>
     </row>
-    <row r="349" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="349" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A349" s="6" t="s">
         <v>75</v>
       </c>
@@ -19017,7 +19020,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="350" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="350" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A350" s="13" t="s">
         <v>217</v>
       </c>
@@ -19066,7 +19069,7 @@
       </c>
       <c r="S350" s="13"/>
     </row>
-    <row r="351" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="351" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A351" s="6" t="s">
         <v>28</v>
       </c>
@@ -19113,7 +19116,7 @@
       </c>
       <c r="S351" s="6"/>
     </row>
-    <row r="352" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="352" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A352" s="11" t="s">
         <v>168</v>
       </c>
@@ -19160,7 +19163,7 @@
       </c>
       <c r="S352" s="11"/>
     </row>
-    <row r="353" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="353" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A353" s="13" t="s">
         <v>169</v>
       </c>
@@ -19209,7 +19212,7 @@
       </c>
       <c r="S353" s="13"/>
     </row>
-    <row r="354" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="354" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A354" s="13" t="s">
         <v>158</v>
       </c>
@@ -19256,7 +19259,7 @@
       </c>
       <c r="S354" s="13"/>
     </row>
-    <row r="355" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="355" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A355" s="6" t="s">
         <v>36</v>
       </c>
@@ -19303,7 +19306,7 @@
       </c>
       <c r="S355" s="6"/>
     </row>
-    <row r="356" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="356" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A356" s="6" t="s">
         <v>49</v>
       </c>
@@ -19350,7 +19353,7 @@
       </c>
       <c r="S356" s="6"/>
     </row>
-    <row r="357" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="357" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A357" s="6" t="s">
         <v>50</v>
       </c>
@@ -19397,7 +19400,7 @@
       </c>
       <c r="S357" s="6"/>
     </row>
-    <row r="358" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="358" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A358" s="6" t="s">
         <v>51</v>
       </c>
@@ -19444,7 +19447,7 @@
       </c>
       <c r="S358" s="6"/>
     </row>
-    <row r="359" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.5">
+    <row r="359" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A359" s="6" t="s">
         <v>86</v>
       </c>
@@ -19491,7 +19494,7 @@
       </c>
       <c r="S359" s="6"/>
     </row>
-    <row r="360" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="360" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A360" s="6" t="s">
         <v>52</v>
       </c>
@@ -19536,7 +19539,7 @@
       </c>
       <c r="S360" s="6"/>
     </row>
-    <row r="361" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="361" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A361" s="6" t="s">
         <v>340</v>
       </c>
@@ -19583,7 +19586,7 @@
       </c>
       <c r="S361" s="6"/>
     </row>
-    <row r="362" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="362" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A362" s="6" t="s">
         <v>71</v>
       </c>
@@ -19628,7 +19631,7 @@
       </c>
       <c r="S362" s="6"/>
     </row>
-    <row r="363" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="363" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A363" s="6" t="s">
         <v>42</v>
       </c>
@@ -19675,7 +19678,7 @@
       </c>
       <c r="S363" s="6"/>
     </row>
-    <row r="364" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="364" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A364" s="6" t="s">
         <v>46</v>
       </c>
@@ -19722,7 +19725,7 @@
       </c>
       <c r="S364" s="6"/>
     </row>
-    <row r="365" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="365" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A365" s="6" t="s">
         <v>47</v>
       </c>
@@ -19767,7 +19770,7 @@
       </c>
       <c r="S365" s="6"/>
     </row>
-    <row r="366" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="366" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A366" s="6" t="s">
         <v>39</v>
       </c>
@@ -19814,7 +19817,7 @@
       </c>
       <c r="S366" s="6"/>
     </row>
-    <row r="367" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="367" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A367" s="11" t="s">
         <v>150</v>
       </c>
@@ -19861,7 +19864,7 @@
       </c>
       <c r="S367" s="13"/>
     </row>
-    <row r="368" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="368" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A368" s="6" t="s">
         <v>150</v>
       </c>
@@ -19908,7 +19911,7 @@
       </c>
       <c r="S368" s="6"/>
     </row>
-    <row r="369" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="369" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A369" s="6" t="s">
         <v>150</v>
       </c>
@@ -19955,7 +19958,7 @@
       </c>
       <c r="S369" s="6"/>
     </row>
-    <row r="370" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="370" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A370" s="6" t="s">
         <v>150</v>
       </c>
@@ -20002,7 +20005,7 @@
       </c>
       <c r="S370" s="6"/>
     </row>
-    <row r="371" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="371" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A371" s="6" t="s">
         <v>74</v>
       </c>
@@ -20049,7 +20052,7 @@
       </c>
       <c r="S371" s="6"/>
     </row>
-    <row r="372" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="372" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A372" s="6" t="s">
         <v>74</v>
       </c>
@@ -20096,7 +20099,7 @@
       </c>
       <c r="S372" s="6"/>
     </row>
-    <row r="373" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="373" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A373" s="6" t="s">
         <v>74</v>
       </c>
@@ -20143,7 +20146,7 @@
       </c>
       <c r="S373" s="6"/>
     </row>
-    <row r="374" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="374" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A374" s="6" t="s">
         <v>78</v>
       </c>
@@ -20188,7 +20191,7 @@
       </c>
       <c r="S374" s="6"/>
     </row>
-    <row r="375" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="375" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A375" s="13" t="s">
         <v>229</v>
       </c>
@@ -20239,7 +20242,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="376" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="376" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A376" s="13" t="s">
         <v>229</v>
       </c>
@@ -20290,7 +20293,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="377" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="377" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A377" s="11" t="s">
         <v>151</v>
       </c>
@@ -20337,7 +20340,7 @@
       </c>
       <c r="S377" s="13"/>
     </row>
-    <row r="378" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="378" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A378" s="11" t="s">
         <v>155</v>
       </c>
@@ -20384,7 +20387,7 @@
       </c>
       <c r="S378" s="13"/>
     </row>
-    <row r="379" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="379" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A379" s="11" t="s">
         <v>153</v>
       </c>
@@ -20433,7 +20436,7 @@
       </c>
       <c r="S379" s="13"/>
     </row>
-    <row r="380" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="380" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A380" s="13" t="s">
         <v>179</v>
       </c>
@@ -20480,7 +20483,7 @@
       </c>
       <c r="S380" s="13"/>
     </row>
-    <row r="381" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="381" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A381" s="6"/>
       <c r="B381" s="6"/>
       <c r="C381" s="7"/>
@@ -20501,7 +20504,7 @@
       <c r="R381" s="13"/>
       <c r="S381" s="6"/>
     </row>
-    <row r="382" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="382" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A382" s="4"/>
       <c r="B382" s="4"/>
       <c r="C382" s="4"/>
@@ -20522,7 +20525,7 @@
       <c r="R382" s="4"/>
       <c r="S382" s="4"/>
     </row>
-    <row r="383" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="383" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A383" s="4"/>
       <c r="B383" s="4"/>
       <c r="C383" s="4"/>
@@ -20543,7 +20546,7 @@
       <c r="R383" s="4"/>
       <c r="S383" s="4"/>
     </row>
-    <row r="384" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="384" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A384" s="4"/>
       <c r="B384" s="4"/>
       <c r="C384" s="4"/>
@@ -20564,7 +20567,7 @@
       <c r="R384" s="4"/>
       <c r="S384" s="4"/>
     </row>
-    <row r="385" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="385" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A385" s="4"/>
       <c r="B385" s="4"/>
       <c r="C385" s="4"/>
@@ -20585,94 +20588,94 @@
       <c r="R385" s="4"/>
       <c r="S385" s="4"/>
     </row>
-    <row r="386" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="386" spans="1:19" x14ac:dyDescent="0.25">
       <c r="O386" s="28"/>
     </row>
-    <row r="387" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="387" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A387" s="4"/>
       <c r="S387" s="4"/>
     </row>
-    <row r="388" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="388" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A388" s="4"/>
       <c r="S388" s="4"/>
     </row>
-    <row r="389" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="389" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A389" s="4"/>
       <c r="S389" s="4"/>
     </row>
-    <row r="390" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="390" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A390" s="4"/>
       <c r="S390" s="4"/>
     </row>
-    <row r="391" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="391" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A391" s="4"/>
       <c r="S391" s="4"/>
     </row>
-    <row r="392" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="392" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A392" s="4"/>
       <c r="S392" s="4"/>
     </row>
-    <row r="393" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="393" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A393" s="4"/>
       <c r="S393" s="4"/>
     </row>
-    <row r="394" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="394" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A394" s="4"/>
       <c r="S394" s="4"/>
     </row>
-    <row r="395" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="395" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A395" s="4"/>
       <c r="S395" s="4"/>
     </row>
-    <row r="396" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="396" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A396" s="4"/>
       <c r="S396" s="4"/>
     </row>
-    <row r="397" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="397" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A397" s="4"/>
       <c r="S397" s="4"/>
     </row>
-    <row r="398" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="398" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A398" s="4"/>
       <c r="S398" s="4"/>
     </row>
-    <row r="399" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="399" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A399" s="4"/>
       <c r="S399" s="4"/>
     </row>
-    <row r="400" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="400" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A400" s="4"/>
       <c r="S400" s="4"/>
     </row>
-    <row r="401" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="401" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A401" s="4"/>
       <c r="S401" s="4"/>
     </row>
-    <row r="402" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="402" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A402" s="4"/>
       <c r="S402" s="4"/>
     </row>
-    <row r="403" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="403" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A403" s="4"/>
       <c r="S403" s="4"/>
     </row>
-    <row r="404" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="404" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A404" s="4"/>
       <c r="S404" s="4"/>
     </row>
-    <row r="405" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="405" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A405" s="4"/>
       <c r="S405" s="4"/>
     </row>
-    <row r="406" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="406" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A406" s="4"/>
       <c r="S406" s="4"/>
     </row>
-    <row r="407" spans="1:19" x14ac:dyDescent="0.5">
+    <row r="407" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A407" s="4"/>
       <c r="S407" s="4"/>
     </row>
-    <row r="408" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="408" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A408" s="4"/>
       <c r="S408" s="4"/>
     </row>
@@ -20762,23 +20765,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0117B9A2-DAC6-A44C-B164-58AB55D11287}">
   <dimension ref="A1:Z57"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.3125" customWidth="1"/>
-    <col min="2" max="2" width="10.1875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.3125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.375" customWidth="1"/>
+    <col min="2" max="2" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.8125" customWidth="1"/>
+    <col min="5" max="5" width="20.875" customWidth="1"/>
     <col min="6" max="6" width="103.5" customWidth="1"/>
-    <col min="7" max="7" width="34.3125" customWidth="1"/>
-    <col min="9" max="9" width="33.1875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="71.3125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.1875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34.375" customWidth="1"/>
+    <col min="9" max="9" width="33.25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="71.375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.25" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="65" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="29" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>474</v>
       </c>
@@ -20786,7 +20789,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>475</v>
       </c>
@@ -20794,7 +20797,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>476</v>
       </c>
@@ -20802,7 +20805,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>477</v>
       </c>
@@ -20810,7 +20813,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>480</v>
       </c>
@@ -20818,7 +20821,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>481</v>
       </c>
@@ -20826,7 +20829,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" s="30" t="s">
         <v>425</v>
       </c>
@@ -20864,7 +20867,7 @@
       <c r="Y9" s="4"/>
       <c r="Z9" s="4"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>471</v>
       </c>
@@ -20930,7 +20933,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>471</v>
       </c>
@@ -20994,7 +20997,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="31" t="s">
         <v>471</v>
       </c>
@@ -21056,7 +21059,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>471</v>
       </c>
@@ -21118,7 +21121,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" s="31" t="s">
         <v>471</v>
       </c>
@@ -21180,7 +21183,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>471</v>
       </c>
@@ -21242,7 +21245,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>471</v>
       </c>
@@ -21302,7 +21305,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>471</v>
       </c>
@@ -21354,7 +21357,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A18" s="31" t="s">
         <v>471</v>
       </c>
@@ -21406,7 +21409,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>471</v>
       </c>
@@ -21458,7 +21461,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20" s="31" t="s">
         <v>471</v>
       </c>
@@ -21508,7 +21511,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>472</v>
       </c>
@@ -21556,7 +21559,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>472</v>
       </c>
@@ -21604,7 +21607,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>472</v>
       </c>
@@ -21652,7 +21655,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>472</v>
       </c>
@@ -21698,7 +21701,7 @@
       </c>
       <c r="Z24" s="4"/>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>472</v>
       </c>
@@ -21744,7 +21747,7 @@
       </c>
       <c r="Z25" s="4"/>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>472</v>
       </c>
@@ -21790,7 +21793,7 @@
       </c>
       <c r="Z26" s="4"/>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>472</v>
       </c>
@@ -21834,7 +21837,7 @@
       </c>
       <c r="Z27" s="4"/>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>472</v>
       </c>
@@ -21878,7 +21881,7 @@
       </c>
       <c r="Z28" s="4"/>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>472</v>
       </c>
@@ -21922,7 +21925,7 @@
       </c>
       <c r="Z29" s="4"/>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>472</v>
       </c>
@@ -21966,7 +21969,7 @@
       </c>
       <c r="Z30" s="4"/>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>472</v>
       </c>
@@ -21989,7 +21992,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A32" s="31" t="s">
         <v>472</v>
       </c>
@@ -22012,7 +22015,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>472</v>
       </c>
@@ -22029,13 +22032,13 @@
         <v>466</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>457</v>
+        <v>488</v>
       </c>
       <c r="G33" s="4" t="s">
         <v>465</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.5">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="31" t="s">
         <v>472</v>
       </c>
@@ -22058,12 +22061,12 @@
         <v>465</v>
       </c>
     </row>
-    <row r="54" spans="3:6" x14ac:dyDescent="0.5">
+    <row r="54" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C54" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="55" spans="3:6" x14ac:dyDescent="0.5">
+    <row r="55" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C55" t="s">
         <v>445</v>
       </c>
@@ -22071,7 +22074,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="56" spans="3:6" x14ac:dyDescent="0.5">
+    <row r="56" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C56" t="s">
         <v>446</v>
       </c>
@@ -22079,7 +22082,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="57" spans="3:6" x14ac:dyDescent="0.5">
+    <row r="57" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C57" t="s">
         <v>443</v>
       </c>
@@ -22098,19 +22101,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7615581-3FCF-FC42-8E0B-B15A61A0919B}">
   <dimension ref="A3:AG55"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.1875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.1875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="29" width="7.8125" customWidth="1"/>
-    <col min="30" max="30" width="14.6875" customWidth="1"/>
-    <col min="32" max="32" width="104.1875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="28.1875" bestFit="1" customWidth="1"/>
+    <col min="6" max="29" width="7.875" customWidth="1"/>
+    <col min="30" max="30" width="14.75" customWidth="1"/>
+    <col min="32" max="32" width="104.25" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="28.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="33"/>
       <c r="B3" s="33"/>
       <c r="C3" s="41" t="s">
@@ -22201,11 +22204,11 @@
         <v>424</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A4" s="60" t="s">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A4" s="61" t="s">
         <v>471</v>
       </c>
-      <c r="B4" s="60" t="s">
+      <c r="B4" s="61" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="4" t="s">
@@ -22249,9 +22252,9 @@
         <v>465</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A5" s="60"/>
-      <c r="B5" s="60"/>
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A5" s="61"/>
+      <c r="B5" s="61"/>
       <c r="C5" s="4" t="s">
         <v>441</v>
       </c>
@@ -22293,9 +22296,9 @@
         <v>465</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A6" s="60"/>
-      <c r="B6" s="60"/>
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A6" s="61"/>
+      <c r="B6" s="61"/>
       <c r="C6" s="4" t="s">
         <v>441</v>
       </c>
@@ -22337,9 +22340,9 @@
         <v>465</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A7" s="60"/>
-      <c r="B7" s="60"/>
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A7" s="61"/>
+      <c r="B7" s="61"/>
       <c r="C7" s="4" t="s">
         <v>444</v>
       </c>
@@ -22381,9 +22384,9 @@
         <v>465</v>
       </c>
     </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A8" s="60"/>
-      <c r="B8" s="61" t="s">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A8" s="61"/>
+      <c r="B8" s="62" t="s">
         <v>29</v>
       </c>
       <c r="C8" s="36" t="s">
@@ -22427,9 +22430,9 @@
         <v>465</v>
       </c>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A9" s="60"/>
-      <c r="B9" s="61"/>
+    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A9" s="61"/>
+      <c r="B9" s="62"/>
       <c r="C9" s="36" t="s">
         <v>442</v>
       </c>
@@ -22471,9 +22474,9 @@
         <v>465</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A10" s="60"/>
-      <c r="B10" s="61"/>
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A10" s="61"/>
+      <c r="B10" s="62"/>
       <c r="C10" s="36" t="s">
         <v>442</v>
       </c>
@@ -22515,11 +22518,11 @@
         <v>465</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A11" s="60" t="s">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A11" s="61" t="s">
         <v>472</v>
       </c>
-      <c r="B11" s="60" t="s">
+      <c r="B11" s="61" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="4" t="s">
@@ -22563,9 +22566,9 @@
         <v>465</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A12" s="60"/>
-      <c r="B12" s="60"/>
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A12" s="61"/>
+      <c r="B12" s="61"/>
       <c r="C12" s="4" t="s">
         <v>433</v>
       </c>
@@ -22607,9 +22610,9 @@
         <v>465</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A13" s="60"/>
-      <c r="B13" s="60"/>
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A13" s="61"/>
+      <c r="B13" s="61"/>
       <c r="C13" s="4" t="s">
         <v>433</v>
       </c>
@@ -22651,9 +22654,9 @@
         <v>465</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A14" s="60"/>
-      <c r="B14" s="60"/>
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A14" s="61"/>
+      <c r="B14" s="61"/>
       <c r="C14" s="4" t="s">
         <v>422</v>
       </c>
@@ -22663,30 +22666,30 @@
       <c r="E14" s="4" t="s">
         <v>423</v>
       </c>
-      <c r="F14" s="51"/>
-      <c r="G14" s="52"/>
-      <c r="H14" s="52"/>
-      <c r="I14" s="52"/>
-      <c r="J14" s="52"/>
-      <c r="K14" s="52"/>
-      <c r="L14" s="52"/>
-      <c r="M14" s="52"/>
-      <c r="N14" s="52"/>
-      <c r="O14" s="52"/>
-      <c r="P14" s="52"/>
-      <c r="Q14" s="52"/>
-      <c r="R14" s="52"/>
-      <c r="S14" s="52"/>
-      <c r="T14" s="52"/>
-      <c r="U14" s="52"/>
-      <c r="V14" s="52"/>
-      <c r="W14" s="52"/>
-      <c r="X14" s="52"/>
-      <c r="Y14" s="52"/>
-      <c r="Z14" s="52"/>
-      <c r="AA14" s="52"/>
-      <c r="AB14" s="52"/>
-      <c r="AC14" s="53"/>
+      <c r="F14" s="52"/>
+      <c r="G14" s="53"/>
+      <c r="H14" s="53"/>
+      <c r="I14" s="53"/>
+      <c r="J14" s="53"/>
+      <c r="K14" s="53"/>
+      <c r="L14" s="53"/>
+      <c r="M14" s="53"/>
+      <c r="N14" s="53"/>
+      <c r="O14" s="53"/>
+      <c r="P14" s="53"/>
+      <c r="Q14" s="53"/>
+      <c r="R14" s="53"/>
+      <c r="S14" s="53"/>
+      <c r="T14" s="53"/>
+      <c r="U14" s="53"/>
+      <c r="V14" s="53"/>
+      <c r="W14" s="53"/>
+      <c r="X14" s="53"/>
+      <c r="Y14" s="53"/>
+      <c r="Z14" s="53"/>
+      <c r="AA14" s="53"/>
+      <c r="AB14" s="53"/>
+      <c r="AC14" s="54"/>
       <c r="AD14" s="35">
         <v>0.2</v>
       </c>
@@ -22697,9 +22700,9 @@
         <v>439</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A15" s="60"/>
-      <c r="B15" s="60"/>
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A15" s="61"/>
+      <c r="B15" s="61"/>
       <c r="C15" s="4" t="s">
         <v>422</v>
       </c>
@@ -22709,30 +22712,30 @@
       <c r="E15" s="4" t="s">
         <v>423</v>
       </c>
-      <c r="F15" s="54"/>
-      <c r="G15" s="55"/>
-      <c r="H15" s="55"/>
-      <c r="I15" s="55"/>
-      <c r="J15" s="55"/>
-      <c r="K15" s="55"/>
-      <c r="L15" s="55"/>
-      <c r="M15" s="55"/>
-      <c r="N15" s="55"/>
-      <c r="O15" s="55"/>
-      <c r="P15" s="55"/>
-      <c r="Q15" s="55"/>
-      <c r="R15" s="55"/>
-      <c r="S15" s="55"/>
-      <c r="T15" s="55"/>
-      <c r="U15" s="55"/>
-      <c r="V15" s="55"/>
-      <c r="W15" s="55"/>
-      <c r="X15" s="55"/>
-      <c r="Y15" s="55"/>
-      <c r="Z15" s="55"/>
-      <c r="AA15" s="55"/>
-      <c r="AB15" s="55"/>
-      <c r="AC15" s="56"/>
+      <c r="F15" s="55"/>
+      <c r="G15" s="56"/>
+      <c r="H15" s="56"/>
+      <c r="I15" s="56"/>
+      <c r="J15" s="56"/>
+      <c r="K15" s="56"/>
+      <c r="L15" s="56"/>
+      <c r="M15" s="56"/>
+      <c r="N15" s="56"/>
+      <c r="O15" s="56"/>
+      <c r="P15" s="56"/>
+      <c r="Q15" s="56"/>
+      <c r="R15" s="56"/>
+      <c r="S15" s="56"/>
+      <c r="T15" s="56"/>
+      <c r="U15" s="56"/>
+      <c r="V15" s="56"/>
+      <c r="W15" s="56"/>
+      <c r="X15" s="56"/>
+      <c r="Y15" s="56"/>
+      <c r="Z15" s="56"/>
+      <c r="AA15" s="56"/>
+      <c r="AB15" s="56"/>
+      <c r="AC15" s="57"/>
       <c r="AD15" s="35">
         <v>0.3</v>
       </c>
@@ -22743,9 +22746,9 @@
         <v>439</v>
       </c>
     </row>
-    <row r="16" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A16" s="60"/>
-      <c r="B16" s="60"/>
+    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A16" s="61"/>
+      <c r="B16" s="61"/>
       <c r="C16" s="4" t="s">
         <v>422</v>
       </c>
@@ -22755,30 +22758,30 @@
       <c r="E16" s="4" t="s">
         <v>423</v>
       </c>
-      <c r="F16" s="54"/>
-      <c r="G16" s="55"/>
-      <c r="H16" s="55"/>
-      <c r="I16" s="55"/>
-      <c r="J16" s="55"/>
-      <c r="K16" s="55"/>
-      <c r="L16" s="55"/>
-      <c r="M16" s="55"/>
-      <c r="N16" s="55"/>
-      <c r="O16" s="55"/>
-      <c r="P16" s="55"/>
-      <c r="Q16" s="55"/>
-      <c r="R16" s="55"/>
-      <c r="S16" s="55"/>
-      <c r="T16" s="55"/>
-      <c r="U16" s="55"/>
-      <c r="V16" s="55"/>
-      <c r="W16" s="55"/>
-      <c r="X16" s="55"/>
-      <c r="Y16" s="55"/>
-      <c r="Z16" s="55"/>
-      <c r="AA16" s="55"/>
-      <c r="AB16" s="55"/>
-      <c r="AC16" s="56"/>
+      <c r="F16" s="55"/>
+      <c r="G16" s="56"/>
+      <c r="H16" s="56"/>
+      <c r="I16" s="56"/>
+      <c r="J16" s="56"/>
+      <c r="K16" s="56"/>
+      <c r="L16" s="56"/>
+      <c r="M16" s="56"/>
+      <c r="N16" s="56"/>
+      <c r="O16" s="56"/>
+      <c r="P16" s="56"/>
+      <c r="Q16" s="56"/>
+      <c r="R16" s="56"/>
+      <c r="S16" s="56"/>
+      <c r="T16" s="56"/>
+      <c r="U16" s="56"/>
+      <c r="V16" s="56"/>
+      <c r="W16" s="56"/>
+      <c r="X16" s="56"/>
+      <c r="Y16" s="56"/>
+      <c r="Z16" s="56"/>
+      <c r="AA16" s="56"/>
+      <c r="AB16" s="56"/>
+      <c r="AC16" s="57"/>
       <c r="AD16" s="35">
         <v>0.1</v>
       </c>
@@ -22789,9 +22792,9 @@
         <v>439</v>
       </c>
     </row>
-    <row r="17" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A17" s="60"/>
-      <c r="B17" s="60"/>
+    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A17" s="61"/>
+      <c r="B17" s="61"/>
       <c r="C17" s="4" t="s">
         <v>438</v>
       </c>
@@ -22801,30 +22804,30 @@
       <c r="E17" s="4" t="s">
         <v>437</v>
       </c>
-      <c r="F17" s="54"/>
-      <c r="G17" s="55"/>
-      <c r="H17" s="55"/>
-      <c r="I17" s="55"/>
-      <c r="J17" s="55"/>
-      <c r="K17" s="55"/>
-      <c r="L17" s="55"/>
-      <c r="M17" s="55"/>
-      <c r="N17" s="55"/>
-      <c r="O17" s="55"/>
-      <c r="P17" s="55"/>
-      <c r="Q17" s="55"/>
-      <c r="R17" s="55"/>
-      <c r="S17" s="55"/>
-      <c r="T17" s="55"/>
-      <c r="U17" s="55"/>
-      <c r="V17" s="55"/>
-      <c r="W17" s="55"/>
-      <c r="X17" s="55"/>
-      <c r="Y17" s="55"/>
-      <c r="Z17" s="55"/>
-      <c r="AA17" s="55"/>
-      <c r="AB17" s="55"/>
-      <c r="AC17" s="56"/>
+      <c r="F17" s="55"/>
+      <c r="G17" s="56"/>
+      <c r="H17" s="56"/>
+      <c r="I17" s="56"/>
+      <c r="J17" s="56"/>
+      <c r="K17" s="56"/>
+      <c r="L17" s="56"/>
+      <c r="M17" s="56"/>
+      <c r="N17" s="56"/>
+      <c r="O17" s="56"/>
+      <c r="P17" s="56"/>
+      <c r="Q17" s="56"/>
+      <c r="R17" s="56"/>
+      <c r="S17" s="56"/>
+      <c r="T17" s="56"/>
+      <c r="U17" s="56"/>
+      <c r="V17" s="56"/>
+      <c r="W17" s="56"/>
+      <c r="X17" s="56"/>
+      <c r="Y17" s="56"/>
+      <c r="Z17" s="56"/>
+      <c r="AA17" s="56"/>
+      <c r="AB17" s="56"/>
+      <c r="AC17" s="57"/>
       <c r="AD17" s="4">
         <v>5</v>
       </c>
@@ -22835,9 +22838,9 @@
         <v>439</v>
       </c>
     </row>
-    <row r="18" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A18" s="60"/>
-      <c r="B18" s="60"/>
+    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A18" s="61"/>
+      <c r="B18" s="61"/>
       <c r="C18" s="4" t="s">
         <v>438</v>
       </c>
@@ -22847,30 +22850,30 @@
       <c r="E18" s="4" t="s">
         <v>437</v>
       </c>
-      <c r="F18" s="54"/>
-      <c r="G18" s="55"/>
-      <c r="H18" s="55"/>
-      <c r="I18" s="55"/>
-      <c r="J18" s="55"/>
-      <c r="K18" s="55"/>
-      <c r="L18" s="55"/>
-      <c r="M18" s="55"/>
-      <c r="N18" s="55"/>
-      <c r="O18" s="55"/>
-      <c r="P18" s="55"/>
-      <c r="Q18" s="55"/>
-      <c r="R18" s="55"/>
-      <c r="S18" s="55"/>
-      <c r="T18" s="55"/>
-      <c r="U18" s="55"/>
-      <c r="V18" s="55"/>
-      <c r="W18" s="55"/>
-      <c r="X18" s="55"/>
-      <c r="Y18" s="55"/>
-      <c r="Z18" s="55"/>
-      <c r="AA18" s="55"/>
-      <c r="AB18" s="55"/>
-      <c r="AC18" s="56"/>
+      <c r="F18" s="55"/>
+      <c r="G18" s="56"/>
+      <c r="H18" s="56"/>
+      <c r="I18" s="56"/>
+      <c r="J18" s="56"/>
+      <c r="K18" s="56"/>
+      <c r="L18" s="56"/>
+      <c r="M18" s="56"/>
+      <c r="N18" s="56"/>
+      <c r="O18" s="56"/>
+      <c r="P18" s="56"/>
+      <c r="Q18" s="56"/>
+      <c r="R18" s="56"/>
+      <c r="S18" s="56"/>
+      <c r="T18" s="56"/>
+      <c r="U18" s="56"/>
+      <c r="V18" s="56"/>
+      <c r="W18" s="56"/>
+      <c r="X18" s="56"/>
+      <c r="Y18" s="56"/>
+      <c r="Z18" s="56"/>
+      <c r="AA18" s="56"/>
+      <c r="AB18" s="56"/>
+      <c r="AC18" s="57"/>
       <c r="AD18" s="4">
         <v>4</v>
       </c>
@@ -22881,9 +22884,9 @@
         <v>439</v>
       </c>
     </row>
-    <row r="19" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A19" s="60"/>
-      <c r="B19" s="60"/>
+    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A19" s="61"/>
+      <c r="B19" s="61"/>
       <c r="C19" s="4" t="s">
         <v>438</v>
       </c>
@@ -22893,30 +22896,30 @@
       <c r="E19" s="4" t="s">
         <v>437</v>
       </c>
-      <c r="F19" s="57"/>
-      <c r="G19" s="58"/>
-      <c r="H19" s="58"/>
-      <c r="I19" s="58"/>
-      <c r="J19" s="58"/>
-      <c r="K19" s="58"/>
-      <c r="L19" s="58"/>
-      <c r="M19" s="58"/>
-      <c r="N19" s="58"/>
-      <c r="O19" s="58"/>
-      <c r="P19" s="58"/>
-      <c r="Q19" s="58"/>
-      <c r="R19" s="58"/>
-      <c r="S19" s="58"/>
-      <c r="T19" s="58"/>
-      <c r="U19" s="58"/>
-      <c r="V19" s="58"/>
-      <c r="W19" s="58"/>
-      <c r="X19" s="58"/>
-      <c r="Y19" s="58"/>
-      <c r="Z19" s="58"/>
-      <c r="AA19" s="58"/>
-      <c r="AB19" s="58"/>
-      <c r="AC19" s="59"/>
+      <c r="F19" s="58"/>
+      <c r="G19" s="59"/>
+      <c r="H19" s="59"/>
+      <c r="I19" s="59"/>
+      <c r="J19" s="59"/>
+      <c r="K19" s="59"/>
+      <c r="L19" s="59"/>
+      <c r="M19" s="59"/>
+      <c r="N19" s="59"/>
+      <c r="O19" s="59"/>
+      <c r="P19" s="59"/>
+      <c r="Q19" s="59"/>
+      <c r="R19" s="59"/>
+      <c r="S19" s="59"/>
+      <c r="T19" s="59"/>
+      <c r="U19" s="59"/>
+      <c r="V19" s="59"/>
+      <c r="W19" s="59"/>
+      <c r="X19" s="59"/>
+      <c r="Y19" s="59"/>
+      <c r="Z19" s="59"/>
+      <c r="AA19" s="59"/>
+      <c r="AB19" s="59"/>
+      <c r="AC19" s="60"/>
       <c r="AD19" s="4">
         <v>6</v>
       </c>
@@ -22927,9 +22930,9 @@
         <v>439</v>
       </c>
     </row>
-    <row r="20" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A20" s="60"/>
-      <c r="B20" s="61" t="s">
+    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A20" s="61"/>
+      <c r="B20" s="62" t="s">
         <v>29</v>
       </c>
       <c r="C20" s="36" t="s">
@@ -22973,9 +22976,9 @@
         <v>465</v>
       </c>
     </row>
-    <row r="21" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A21" s="60"/>
-      <c r="B21" s="61"/>
+    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A21" s="61"/>
+      <c r="B21" s="62"/>
       <c r="C21" s="36" t="s">
         <v>434</v>
       </c>
@@ -23017,9 +23020,9 @@
         <v>465</v>
       </c>
     </row>
-    <row r="22" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="A22" s="60"/>
-      <c r="B22" s="61"/>
+    <row r="22" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A22" s="61"/>
+      <c r="B22" s="62"/>
       <c r="C22" s="36" t="s">
         <v>434</v>
       </c>
@@ -23061,7 +23064,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="27" spans="1:33" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:33" x14ac:dyDescent="0.25">
       <c r="B27" s="4"/>
       <c r="C27" s="30" t="s">
         <v>484</v>
@@ -23146,8 +23149,8 @@
       </c>
       <c r="AD27" s="42"/>
     </row>
-    <row r="28" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="B28" s="60" t="s">
+    <row r="28" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="B28" s="61" t="s">
         <v>21</v>
       </c>
       <c r="C28" s="40" t="s">
@@ -23185,8 +23188,8 @@
       <c r="AC28" s="32"/>
       <c r="AD28" s="43"/>
     </row>
-    <row r="29" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="B29" s="60"/>
+    <row r="29" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="B29" s="61"/>
       <c r="C29" s="40" t="s">
         <v>34</v>
       </c>
@@ -23222,8 +23225,8 @@
       <c r="AC29" s="32"/>
       <c r="AD29" s="43"/>
     </row>
-    <row r="30" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="B30" s="60"/>
+    <row r="30" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="B30" s="61"/>
       <c r="C30" s="40" t="s">
         <v>99</v>
       </c>
@@ -23259,8 +23262,8 @@
       <c r="AC30" s="32"/>
       <c r="AD30" s="43"/>
     </row>
-    <row r="31" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="B31" s="60"/>
+    <row r="31" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="B31" s="61"/>
       <c r="C31" s="40" t="s">
         <v>132</v>
       </c>
@@ -23296,8 +23299,8 @@
       <c r="AC31" s="32"/>
       <c r="AD31" s="43"/>
     </row>
-    <row r="32" spans="1:33" x14ac:dyDescent="0.5">
-      <c r="B32" s="60"/>
+    <row r="32" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="B32" s="61"/>
       <c r="C32" s="40" t="s">
         <v>40</v>
       </c>
@@ -23333,8 +23336,8 @@
       <c r="AC32" s="32"/>
       <c r="AD32" s="43"/>
     </row>
-    <row r="33" spans="2:30" x14ac:dyDescent="0.5">
-      <c r="B33" s="60"/>
+    <row r="33" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="B33" s="61"/>
       <c r="C33" s="40" t="s">
         <v>44</v>
       </c>
@@ -23370,8 +23373,8 @@
       <c r="AC33" s="32"/>
       <c r="AD33" s="43"/>
     </row>
-    <row r="34" spans="2:30" x14ac:dyDescent="0.5">
-      <c r="B34" s="60"/>
+    <row r="34" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="B34" s="61"/>
       <c r="C34" s="40" t="s">
         <v>221</v>
       </c>
@@ -23407,8 +23410,8 @@
       <c r="AC34" s="32"/>
       <c r="AD34" s="43"/>
     </row>
-    <row r="35" spans="2:30" x14ac:dyDescent="0.5">
-      <c r="B35" s="60"/>
+    <row r="35" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="B35" s="61"/>
       <c r="C35" s="40" t="s">
         <v>56</v>
       </c>
@@ -23444,7 +23447,7 @@
       <c r="AC35" s="32"/>
       <c r="AD35" s="43"/>
     </row>
-    <row r="37" spans="2:30" x14ac:dyDescent="0.5">
+    <row r="37" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B37" s="4"/>
       <c r="C37" s="30" t="s">
         <v>484</v>
@@ -23528,8 +23531,8 @@
         <v>46023</v>
       </c>
     </row>
-    <row r="38" spans="2:30" x14ac:dyDescent="0.5">
-      <c r="B38" s="60" t="s">
+    <row r="38" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="B38" s="61" t="s">
         <v>29</v>
       </c>
       <c r="C38" s="40" t="s">
@@ -23566,8 +23569,8 @@
       <c r="AB38" s="32"/>
       <c r="AC38" s="32"/>
     </row>
-    <row r="39" spans="2:30" x14ac:dyDescent="0.5">
-      <c r="B39" s="60"/>
+    <row r="39" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="B39" s="61"/>
       <c r="C39" s="40" t="s">
         <v>34</v>
       </c>
@@ -23602,8 +23605,8 @@
       <c r="AB39" s="32"/>
       <c r="AC39" s="32"/>
     </row>
-    <row r="40" spans="2:30" x14ac:dyDescent="0.5">
-      <c r="B40" s="60"/>
+    <row r="40" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="B40" s="61"/>
       <c r="C40" s="40" t="s">
         <v>99</v>
       </c>
@@ -23638,8 +23641,8 @@
       <c r="AB40" s="32"/>
       <c r="AC40" s="32"/>
     </row>
-    <row r="41" spans="2:30" x14ac:dyDescent="0.5">
-      <c r="B41" s="60"/>
+    <row r="41" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="B41" s="61"/>
       <c r="C41" s="40" t="s">
         <v>132</v>
       </c>
@@ -23674,8 +23677,8 @@
       <c r="AB41" s="32"/>
       <c r="AC41" s="32"/>
     </row>
-    <row r="42" spans="2:30" x14ac:dyDescent="0.5">
-      <c r="B42" s="60"/>
+    <row r="42" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="B42" s="61"/>
       <c r="C42" s="40" t="s">
         <v>40</v>
       </c>
@@ -23710,8 +23713,8 @@
       <c r="AB42" s="32"/>
       <c r="AC42" s="32"/>
     </row>
-    <row r="43" spans="2:30" x14ac:dyDescent="0.5">
-      <c r="B43" s="60"/>
+    <row r="43" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="B43" s="61"/>
       <c r="C43" s="40" t="s">
         <v>44</v>
       </c>
@@ -23746,8 +23749,8 @@
       <c r="AB43" s="32"/>
       <c r="AC43" s="32"/>
     </row>
-    <row r="44" spans="2:30" x14ac:dyDescent="0.5">
-      <c r="B44" s="60"/>
+    <row r="44" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="B44" s="61"/>
       <c r="C44" s="40" t="s">
         <v>221</v>
       </c>
@@ -23782,8 +23785,8 @@
       <c r="AB44" s="32"/>
       <c r="AC44" s="32"/>
     </row>
-    <row r="45" spans="2:30" x14ac:dyDescent="0.5">
-      <c r="B45" s="60"/>
+    <row r="45" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="B45" s="61"/>
       <c r="C45" s="40" t="s">
         <v>56</v>
       </c>
@@ -23818,7 +23821,7 @@
       <c r="AB45" s="32"/>
       <c r="AC45" s="32"/>
     </row>
-    <row r="47" spans="2:30" x14ac:dyDescent="0.5">
+    <row r="47" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B47" s="4"/>
       <c r="C47" s="30" t="s">
         <v>484</v>
@@ -23902,8 +23905,8 @@
         <v>46023</v>
       </c>
     </row>
-    <row r="48" spans="2:30" x14ac:dyDescent="0.5">
-      <c r="B48" s="62" t="s">
+    <row r="48" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="B48" s="51" t="s">
         <v>487</v>
       </c>
       <c r="C48" s="40" t="s">
@@ -23940,8 +23943,8 @@
       <c r="AB48" s="32"/>
       <c r="AC48" s="32"/>
     </row>
-    <row r="49" spans="2:29" x14ac:dyDescent="0.5">
-      <c r="B49" s="62"/>
+    <row r="49" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B49" s="51"/>
       <c r="C49" s="40" t="s">
         <v>34</v>
       </c>
@@ -23976,8 +23979,8 @@
       <c r="AB49" s="32"/>
       <c r="AC49" s="32"/>
     </row>
-    <row r="50" spans="2:29" x14ac:dyDescent="0.5">
-      <c r="B50" s="62"/>
+    <row r="50" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B50" s="51"/>
       <c r="C50" s="40" t="s">
         <v>99</v>
       </c>
@@ -24012,8 +24015,8 @@
       <c r="AB50" s="32"/>
       <c r="AC50" s="32"/>
     </row>
-    <row r="51" spans="2:29" x14ac:dyDescent="0.5">
-      <c r="B51" s="62"/>
+    <row r="51" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B51" s="51"/>
       <c r="C51" s="40" t="s">
         <v>132</v>
       </c>
@@ -24048,8 +24051,8 @@
       <c r="AB51" s="32"/>
       <c r="AC51" s="32"/>
     </row>
-    <row r="52" spans="2:29" x14ac:dyDescent="0.5">
-      <c r="B52" s="62"/>
+    <row r="52" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B52" s="51"/>
       <c r="C52" s="40" t="s">
         <v>40</v>
       </c>
@@ -24084,8 +24087,8 @@
       <c r="AB52" s="32"/>
       <c r="AC52" s="32"/>
     </row>
-    <row r="53" spans="2:29" x14ac:dyDescent="0.5">
-      <c r="B53" s="62"/>
+    <row r="53" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B53" s="51"/>
       <c r="C53" s="40" t="s">
         <v>44</v>
       </c>
@@ -24120,8 +24123,8 @@
       <c r="AB53" s="32"/>
       <c r="AC53" s="32"/>
     </row>
-    <row r="54" spans="2:29" x14ac:dyDescent="0.5">
-      <c r="B54" s="62"/>
+    <row r="54" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B54" s="51"/>
       <c r="C54" s="40" t="s">
         <v>221</v>
       </c>
@@ -24156,8 +24159,8 @@
       <c r="AB54" s="32"/>
       <c r="AC54" s="32"/>
     </row>
-    <row r="55" spans="2:29" x14ac:dyDescent="0.5">
-      <c r="B55" s="62"/>
+    <row r="55" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B55" s="51"/>
       <c r="C55" s="40" t="s">
         <v>56</v>
       </c>

</xml_diff>